<commit_message>
TEST voor ronde 2
</commit_message>
<xml_diff>
--- a/Questions - Round 2.xlsx
+++ b/Questions - Round 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{6B9D40C8-13C7-40B1-9849-545052FB2826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7254AC0F-27B2-474E-8FC8-95BBE3EEAA21}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{6B9D40C8-13C7-40B1-9849-545052FB2826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15D26AFE-C262-4916-8B00-B169BE6A6A18}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN" sheetId="1" r:id="rId1"/>
@@ -192,7 +192,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="76">
   <si>
     <t>type</t>
   </si>
@@ -224,9 +224,6 @@
     <t>single</t>
   </si>
   <si>
-    <t>What does sustainability in everyday work mean most of all?</t>
-  </si>
-  <si>
     <t>Single choice</t>
   </si>
   <si>
@@ -251,9 +248,6 @@
     <t>multiple</t>
   </si>
   <si>
-    <t>Which goals fit the “Zero in Focus” idea?</t>
-  </si>
-  <si>
     <t>Multiple choice</t>
   </si>
   <si>
@@ -423,6 +417,9 @@
   </si>
   <si>
     <t>Le concept « Zero in Focus » combine les objectifs liés au climat, à la sécurité et à l’intégrité. La formation n’est pas un objectif du programme « Zero ».</t>
+  </si>
+  <si>
+    <t>TEST</t>
   </si>
 </sst>
 </file>
@@ -943,57 +940,57 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1052,57 +1049,57 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1172,57 +1169,57 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1281,57 +1278,57 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1353,7 +1350,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1361,32 +1358,32 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
@@ -1394,7 +1391,7 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>